<commit_message>
Feat: Se agrega Dashboard de KPIs con Tabla y Grafico Dinamico
</commit_message>
<xml_diff>
--- a/Semana_01_Excel_Higiene/ventas_limpias.xlsx
+++ b/Semana_01_Excel_Higiene/ventas_limpias.xlsx
@@ -8,19 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arnol\Desktop\RUTA_DATA_ANALYTICS\Semana_01_Excel_Higiene\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59FAF74F-FF41-4FB2-9C95-4390A69F80BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FAF9C3F-2C24-4301-A937-7A985CD351DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{0311E330-2CB2-4936-8C96-3E3D1504E555}"/>
   </bookViews>
   <sheets>
-    <sheet name="ventas_sucias" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard_KPIs" sheetId="2" r:id="rId1"/>
+    <sheet name="ventas_sucias" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <pivotCaches>
+    <pivotCache cacheId="7" r:id="rId3"/>
+  </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -46,9 +50,6 @@
     <t>Laptop</t>
   </si>
   <si>
-    <t>850.00</t>
-  </si>
-  <si>
     <t>Completado</t>
   </si>
   <si>
@@ -58,18 +59,12 @@
     <t>TECLADO</t>
   </si>
   <si>
-    <t>45.00</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Carlos  Sosa </t>
   </si>
   <si>
     <t>Mouse</t>
   </si>
   <si>
-    <t>25.0</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Pendiente </t>
   </si>
   <si>
@@ -85,9 +80,6 @@
     <t>Monitor</t>
   </si>
   <si>
-    <t>220.00</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Cancelado</t>
   </si>
   <si>
@@ -116,13 +108,27 @@
   </si>
   <si>
     <t>Cancelado</t>
+  </si>
+  <si>
+    <t>Etiquetas de fila</t>
+  </si>
+  <si>
+    <t>Total general</t>
+  </si>
+  <si>
+    <t>Suma de Monto_USD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <numFmts count="3">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -599,9 +605,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -647,7 +661,71 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="21">
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -658,6 +736,1221 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[ventas_limpias.xlsx]Dashboard_KPIs!TablaDinámica1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-AR"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard_KPIs!$B$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard_KPIs!$A$4:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mouse</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>TECLADO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard_KPIs!$B$4:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C71C-4B6E-939A-12E2EA4E8179}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="309982736"/>
+        <c:axId val="308960208"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="309982736"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="308960208"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="308960208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="309982736"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-AR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>445770</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>262890</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7612A11-C3A7-A107-EF87-A53B03CCF96F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Arnoldo Coy" refreshedDate="46234.947724189813" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="5" xr:uid="{12E25725-7959-44DD-84D0-9AAEA721B98F}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:I6" sheet="ventas_sucias"/>
+  </cacheSource>
+  <cacheFields count="9">
+    <cacheField name="ID_Cliente" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="101" maxValue="105"/>
+    </cacheField>
+    <cacheField name="Nombre_Cliente" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Fecha" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-01-15T00:00:00" maxDate="2026-02-11T00:00:00"/>
+    </cacheField>
+    <cacheField name="Producto" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Laptop"/>
+        <s v="TECLADO"/>
+        <s v="Mouse"/>
+        <s v="Monitor"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Monto_USD" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="25" maxValue="850"/>
+    </cacheField>
+    <cacheField name="Estado" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Nombre_Limpio" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Producto_Limpio" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Estado_Limpio" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="5">
+  <r>
+    <n v="101"/>
+    <s v="  Pedro Perez "/>
+    <d v="2026-01-15T00:00:00"/>
+    <x v="0"/>
+    <n v="850"/>
+    <s v="Completado"/>
+    <s v="Pedro Perez"/>
+    <s v="LAPTOP"/>
+    <s v="Completado"/>
+  </r>
+  <r>
+    <n v="102"/>
+    <s v="Maria Gomez"/>
+    <d v="2026-01-15T00:00:00"/>
+    <x v="1"/>
+    <n v="45"/>
+    <s v="Completado"/>
+    <s v="Maria Gomez"/>
+    <s v="TECLADO"/>
+    <s v="Completado"/>
+  </r>
+  <r>
+    <n v="103"/>
+    <s v=" Carlos  Sosa "/>
+    <d v="2026-02-01T00:00:00"/>
+    <x v="2"/>
+    <n v="25"/>
+    <s v=" Pendiente "/>
+    <s v="Carlos Sosa"/>
+    <s v="MOUSE"/>
+    <s v="Pendiente"/>
+  </r>
+  <r>
+    <n v="104"/>
+    <s v="Ana Rodriguez"/>
+    <d v="2026-02-02T00:00:00"/>
+    <x v="0"/>
+    <n v="850"/>
+    <s v="Completado"/>
+    <s v="Ana Rodriguez"/>
+    <s v="LAPTOP"/>
+    <s v="Completado"/>
+  </r>
+  <r>
+    <n v="105"/>
+    <s v="Luis Hernandez"/>
+    <d v="2026-02-10T00:00:00"/>
+    <x v="3"/>
+    <n v="220"/>
+    <s v=" Cancelado"/>
+    <s v="Luis Hernandez"/>
+    <s v="MONITOR"/>
+    <s v="Cancelado"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2A0A4804-0CCB-4448-8B4F-D156B4234FD9}" name="TablaDinámica1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de Monto_USD" fld="4" baseField="0" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="20">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="19">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="18">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="17">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -976,17 +2269,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C223BF-55AA-45DE-A4DE-51D487C8686B}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7D90594-7B92-49A6-A615-6C5918045A48}">
+  <dimension ref="A3:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="13.76171875" customWidth="1"/>
-    <col min="9" max="9" width="12.09375" customWidth="1"/>
+    <col min="1" max="1" width="15.83984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.41796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1990</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C223BF-55AA-45DE-A4DE-51D487C8686B}">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="2" max="2" width="19.83984375" customWidth="1"/>
+    <col min="5" max="5" width="10.9453125" style="5"/>
+    <col min="7" max="7" width="13.578125" customWidth="1"/>
+    <col min="8" max="8" width="13.734375" customWidth="1"/>
+    <col min="9" max="9" width="12.1015625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -999,23 +2357,23 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>101</v>
       </c>
@@ -1028,137 +2386,140 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="7">
+        <v>850</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1">
         <v>46037</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="E3" s="5">
+        <v>45</v>
       </c>
       <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>10</v>
       </c>
-      <c r="H3" t="s">
-        <v>11</v>
-      </c>
       <c r="I3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1">
         <v>46054</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="E4" s="5">
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1">
         <v>46055</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="5">
+        <v>850</v>
+      </c>
+      <c r="F5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1">
         <v>46063</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="E6" s="5">
+        <v>220</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>31</v>
-      </c>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="E7" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>